<commit_message>
UserManagement and Alert Management Testcases
</commit_message>
<xml_diff>
--- a/Common Utils/login.xlsx
+++ b/Common Utils/login.xlsx
@@ -440,16 +440,16 @@
         <v>Verify that the user can log in successfully with valid credentials.</v>
       </c>
       <c r="D2" t="str" xml:space="preserve">
-        <v xml:space="preserve"> The application is deployed and accessible._x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve"> The application is deployed and accessible._x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 - Valid credentials are stored in .env.</v>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Navigate to the login page._x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-2. Enter valid username and password._x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">1. Navigate to the login page._x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+2. Enter valid username and password._x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 3. Click the login button.</v>
       </c>
       <c r="F2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Username: VALID_USERNAME_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">Username: VALID_USERNAME_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Password: VALID_PASSWORD</v>
       </c>
       <c r="G2" t="str">
@@ -473,14 +473,14 @@
         <v>Verify the CSV file based on customedate.</v>
       </c>
       <c r="E3" t="str" xml:space="preserve">
-        <v xml:space="preserve">open the url_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-Enter the userName and Password_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-Enter Captcha_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">open the url_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+Enter the userName and Password_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+Enter Captcha_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Click on the sign in button</v>
       </c>
       <c r="F3" t="str" xml:space="preserve">
-        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Password:xxxx</v>
       </c>
       <c r="G3" t="str">
@@ -545,7 +545,7 @@
     </row>
     <row r="8" xml:space="preserve">
       <c r="E8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Click on the DownLoad button_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">Click on the DownLoad button_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 </v>
       </c>
       <c r="G8" t="str">
@@ -577,13 +577,13 @@
         <v>Verify the CSV file based on timeperiod</v>
       </c>
       <c r="E10" t="str" xml:space="preserve">
-        <v xml:space="preserve">1.Navigate to the login page _x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-2.Enter the User Name and Password_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">1.Navigate to the login page _x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+2.Enter the User Name and Password_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 3.Enter the captcha</v>
       </c>
       <c r="F10" t="str" xml:space="preserve">
-        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Password:xxxx</v>
       </c>
       <c r="G10" t="str">
@@ -676,13 +676,13 @@
         <v>Verify the snapshot file based on timeperiod</v>
       </c>
       <c r="E17" t="str" xml:space="preserve">
-        <v xml:space="preserve">1.Navigate to the login page _x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-2.Enter the User Name and Password_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">1.Navigate to the login page _x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+2.Enter the User Name and Password_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 3.Enter the captcha</v>
       </c>
       <c r="F17" t="str" xml:space="preserve">
-        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Password:xxxx</v>
       </c>
       <c r="G17" t="str">
@@ -780,14 +780,14 @@
         <v>Verify the Mandetory fields in Alert Management module</v>
       </c>
       <c r="E25" t="str" xml:space="preserve">
-        <v xml:space="preserve">open the url_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-Enter the userName and Password_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-Enter Captcha_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">open the url_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+Enter the userName and Password_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+Enter Captcha_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Click on the sign in button</v>
       </c>
       <c r="F25" t="str" xml:space="preserve">
-        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Password:xxxx</v>
       </c>
       <c r="G25" t="str">
@@ -858,15 +858,15 @@
         <v>Verify Alerts History</v>
       </c>
       <c r="E30" t="str" xml:space="preserve">
-        <v xml:space="preserve">_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-open the url_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-Enter the userName and Password_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-Enter Captcha_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+open the url_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+Enter the userName and Password_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+Enter Captcha_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Click on the sign in button</v>
       </c>
       <c r="F30" t="str" xml:space="preserve">
-        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Password:xxxx</v>
       </c>
       <c r="G30" t="str">
@@ -953,18 +953,18 @@
         <v>The user account is created with critical and warning checkboxes enabled and access to the Alarm Setup module. In this module, roles for alert and warning messages can be assigned to selected devices. Data can then be sent via Postman with the assigned roles for critical and warning messages for a particular device.</v>
       </c>
       <c r="E37" t="str" xml:space="preserve">
-        <v xml:space="preserve">Navigate to the homepage_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-Click on the UserManagement_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">Navigate to the homepage_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+Click on the UserManagement_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Search based on user name</v>
       </c>
       <c r="F37" t="str" xml:space="preserve">
-        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Password:xxxx</v>
       </c>
       <c r="G37" t="str" xml:space="preserve">
-        <v xml:space="preserve">Home page should be dispayed_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-Usermanagement Page should be displayed _x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">Home page should be dispayed_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+Usermanagement Page should be displayed _x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Eneter the user Name</v>
       </c>
       <c r="H37" t="str">
@@ -984,12 +984,12 @@
     </row>
     <row r="39" xml:space="preserve">
       <c r="E39" t="str" xml:space="preserve">
-        <v xml:space="preserve">Again login in to the our credentials_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">Again login in to the our credentials_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 1.Navigate the Home Page</v>
       </c>
       <c r="F39" t="str" xml:space="preserve">
-        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Password:xxxx</v>
       </c>
       <c r="G39" t="str">
@@ -1089,9 +1089,9 @@
     </row>
     <row r="48" xml:space="preserve">
       <c r="E48" t="str" xml:space="preserve">
-        <v xml:space="preserve">go to the Email_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-Enter userName_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-password_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">go to the Email_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+Enter userName_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+password_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 click on sign in button</v>
       </c>
       <c r="G48" t="str">
@@ -1123,25 +1123,25 @@
         <v>The user is disabled with critical and warning checkboxes enabled and access to the Alarm Setup module. In this module, roles for alert and warning messages can be assigned to selected devices. Data can then be sent via Postman with the assigned roles for critical and warning messages for a particular device.</v>
       </c>
       <c r="E50" t="str" xml:space="preserve">
-        <v xml:space="preserve">Navigate to the homepage_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-Click on the UserManagement_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">Navigate to the homepage_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+Click on the UserManagement_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Search based on user name</v>
       </c>
       <c r="F50" t="str" xml:space="preserve">
-        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Password:xxxx</v>
       </c>
       <c r="G50" t="str" xml:space="preserve">
-        <v xml:space="preserve">Home page should be dispayed_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-Usermanagement Page should be displayed _x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">Home page should be dispayed_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+Usermanagement Page should be displayed _x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Eneter the user Name</v>
       </c>
       <c r="H50" t="str">
         <v>as Expected</v>
       </c>
       <c r="I50" t="str">
-        <v>Fail</v>
+        <v>Pass</v>
       </c>
     </row>
     <row r="51">
@@ -1157,12 +1157,12 @@
     </row>
     <row r="52" xml:space="preserve">
       <c r="E52" t="str" xml:space="preserve">
-        <v xml:space="preserve">Again login in to the our credentials_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">Again login in to the our credentials_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 1.Navigate the Home Page</v>
       </c>
       <c r="F52" t="str" xml:space="preserve">
-        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">URL: http://staging.dgtrak.online/_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+UseName:xxxxx_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 Password:xxxx</v>
       </c>
       <c r="G52" t="str">
@@ -1251,9 +1251,9 @@
     </row>
     <row r="60" xml:space="preserve">
       <c r="E60" t="str" xml:space="preserve">
-        <v xml:space="preserve">go to the Email_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-Enter userName_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
-password_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">go to the Email_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+Enter userName_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
+password_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_
 click on sign in button</v>
       </c>
       <c r="G60" t="str">
@@ -1308,10 +1308,10 @@
         <v>TC-002</v>
       </c>
       <c r="B3" t="str">
-        <v>user edit</v>
+        <v>roles creation</v>
       </c>
       <c r="C3" t="str">
-        <v>user edit</v>
+        <v>roles creation</v>
       </c>
       <c r="D3" t="str">
         <v>Pass</v>
@@ -1322,10 +1322,10 @@
         <v>TC-003</v>
       </c>
       <c r="B4" t="str">
-        <v>usermandetory fields</v>
+        <v>sorting order</v>
       </c>
       <c r="C4" t="str">
-        <v>usermandetory fileds</v>
+        <v>sorting order</v>
       </c>
       <c r="D4" t="str">
         <v>Pass</v>
@@ -1336,13 +1336,13 @@
         <v>TC-004</v>
       </c>
       <c r="B5" t="str">
-        <v>roles creation</v>
+        <v>usermandetory fields</v>
       </c>
       <c r="C5" t="str">
-        <v>roles creation</v>
+        <v>usermandetory fields</v>
       </c>
       <c r="D5" t="str">
-        <v>Pass</v>
+        <v>Fail</v>
       </c>
     </row>
   </sheetData>

</xml_diff>